<commit_message>
Add OFL license file and unit test for HrPayrollPdfRenderer
- Created a new OFL.txt file for the Be Vietnam Pro font license.
- Added a unit test for HrPayrollPdfRenderer to verify PDF generation for Vietnamese payroll.
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/hr/templates/labor-book-template.xlsx
+++ b/backend/src/main/resources/hr/templates/labor-book-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SO_QUAN_LY_LAO_DONG" sheetId="1" r:id="R3044d4976cf04744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SO_QUAN_LY_LAO_DONG" sheetId="1" r:id="Ra3d14fd3f679400b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
     <x:numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <x:numFmt numFmtId="200" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -58,6 +58,12 @@
       <x:sz val="13"/>
       <x:name val="Times New Roman"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Times New Roman"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -179,7 +185,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="42">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyAlignment="1">
       <x:alignment horizontal="left"/>
@@ -297,6 +303,57 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="14" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="49" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -589,31 +646,32 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <x:col min="3" max="3" width="26" customWidth="1"/>
-    <x:col min="4" max="4" width="9.28515625" customWidth="1"/>
-    <x:col min="5" max="5" width="16" customWidth="1"/>
-    <x:col min="6" max="6" width="10" customWidth="1"/>
-    <x:col min="7" max="7" width="42" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="16.7109375" customWidth="1"/>
-    <x:col min="9" max="9" width="16" customWidth="1"/>
-    <x:col min="10" max="10" width="10" customWidth="1"/>
-    <x:col min="11" max="11" width="24" customWidth="1"/>
-    <x:col min="12" max="12" width="20" customWidth="1"/>
+    <x:col min="1" max="1" width="5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="13" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="11" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="13" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="13" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="16" customWidth="1"/>
-    <x:col min="18" max="18" width="14.85546875" customWidth="1"/>
-    <x:col min="19" max="19" width="7.28515625" customWidth="1"/>
-    <x:col min="20" max="20" width="12" customWidth="1"/>
-    <x:col min="21" max="21" width="9.140625" customWidth="1"/>
-    <x:col min="22" max="22" width="10" customWidth="1"/>
-    <x:col min="23" max="23" width="11.42578125" customWidth="1"/>
-    <x:col min="24" max="24" width="16" hidden="0" customWidth="1"/>
-    <x:col min="25" max="25" width="16" hidden="0" customWidth="1"/>
-    <x:col min="26" max="26" width="34" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="13" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="13" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="15" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="13" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="12" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="12" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="12" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="16" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="18" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="32" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="9" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -644,172 +702,172 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="5" ht="22.5" customHeight="1">
-      <x:c r="A5" s="4" t="inlineStr">
+    <x:row r="5" ht="34" customHeight="1">
+      <x:c r="A5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">STT</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="4" t="inlineStr">
+      <x:c r="B5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">M số</x:t>
         </x:is>
       </x:c>
-      <x:c r="C5" s="4" t="inlineStr">
+      <x:c r="C5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Họ và tên</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="4" t="inlineStr">
+      <x:c r="D5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Giới tính</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="4" t="inlineStr">
+      <x:c r="E5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Ngày tháng năm sinh</x:t>
         </x:is>
       </x:c>
-      <x:c r="F5" s="4" t="inlineStr">
+      <x:c r="F5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Quốc tịch</x:t>
         </x:is>
       </x:c>
-      <x:c r="G5" s="4" t="inlineStr">
+      <x:c r="G5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Nơi cư trú</x:t>
         </x:is>
       </x:c>
-      <x:c r="H5" s="5" t="inlineStr">
+      <x:c r="H5" s="43" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Số thẻ CCCD hoặc CMND hoặc hộ chiếu</x:t>
         </x:is>
       </x:c>
-      <x:c r="I5" s="4" t="inlineStr">
+      <x:c r="I5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Trình độ chuyên môn kỹ thuật</x:t>
         </x:is>
       </x:c>
-      <x:c r="J5" s="4" t="inlineStr">
+      <x:c r="J5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Bậc trình độ kỹ năng nghề</x:t>
         </x:is>
       </x:c>
-      <x:c r="K5" s="4" t="inlineStr">
+      <x:c r="K5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Vị trí làm việc</x:t>
         </x:is>
       </x:c>
-      <x:c r="L5" s="4" t="inlineStr">
+      <x:c r="L5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Loại hợp đồng lao động</x:t>
         </x:is>
       </x:c>
-      <x:c r="M5" s="6" t="inlineStr">
+      <x:c r="M5" s="44" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Thời điểm bắt đầu làm việc</x:t>
         </x:is>
       </x:c>
-      <x:c r="N5" s="4" t="inlineStr">
+      <x:c r="N5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Tham gia bảo hiểm</x:t>
         </x:is>
       </x:c>
-      <x:c r="O5" s="7" t="n"/>
-      <x:c r="P5" s="8" t="n"/>
-      <x:c r="Q5" s="9" t="inlineStr">
+      <x:c r="O5" s="55" t="n"/>
+      <x:c r="P5" s="56" t="n"/>
+      <x:c r="Q5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Tiền lương</x:t>
         </x:is>
       </x:c>
-      <x:c r="R5" s="9" t="inlineStr">
+      <x:c r="R5" s="47" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Phụ cấp</x:t>
         </x:is>
       </x:c>
-      <x:c r="S5" s="4" t="inlineStr">
+      <x:c r="S5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Nâng bậc, nâng lương</x:t>
         </x:is>
       </x:c>
-      <x:c r="T5" s="4" t="inlineStr">
+      <x:c r="T5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Số ngày nghỉ trong năm</x:t>
         </x:is>
       </x:c>
-      <x:c r="U5" s="4" t="inlineStr">
+      <x:c r="U5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Số giờ làm thêm</x:t>
         </x:is>
       </x:c>
-      <x:c r="V5" s="4" t="inlineStr">
+      <x:c r="V5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Hưởng chế độ BHXH, BHYT, BHTN</x:t>
         </x:is>
       </x:c>
-      <x:c r="W5" s="4" t="inlineStr">
+      <x:c r="W5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Học nghề, đào tạo, bồi dưỡng, nâng cao trình độ kỹ năng nghề</x:t>
         </x:is>
       </x:c>
-      <x:c r="X5" s="4" t="inlineStr">
+      <x:c r="X5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Kỷ luật lao động, trách nhiệm vật chất</x:t>
         </x:is>
       </x:c>
-      <x:c r="Y5" s="4" t="inlineStr">
+      <x:c r="Y5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Tai nạn lao động, bệnh nghề nghiệp</x:t>
         </x:is>
       </x:c>
-      <x:c r="Z5" s="4" t="inlineStr">
+      <x:c r="Z5" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Thời điểm chấm dứt hợp đồng lao động và lý do</x:t>
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="6" ht="123.75" customHeight="1">
-      <x:c r="A6" s="10" t="n"/>
-      <x:c r="B6" s="10" t="n"/>
-      <x:c r="C6" s="10" t="n"/>
-      <x:c r="D6" s="10" t="n"/>
-      <x:c r="E6" s="10" t="n"/>
-      <x:c r="F6" s="10" t="n"/>
-      <x:c r="G6" s="10" t="n"/>
-      <x:c r="H6" s="10" t="n"/>
-      <x:c r="I6" s="10" t="n"/>
-      <x:c r="J6" s="10" t="n"/>
-      <x:c r="K6" s="10" t="n"/>
-      <x:c r="L6" s="10" t="n"/>
-      <x:c r="M6" s="10" t="n"/>
-      <x:c r="N6" s="4" t="inlineStr">
+    <x:row r="6" ht="82" customHeight="1">
+      <x:c r="A6" s="57" t="n"/>
+      <x:c r="B6" s="57" t="n"/>
+      <x:c r="C6" s="57" t="n"/>
+      <x:c r="D6" s="57" t="n"/>
+      <x:c r="E6" s="57" t="n"/>
+      <x:c r="F6" s="57" t="n"/>
+      <x:c r="G6" s="57" t="n"/>
+      <x:c r="H6" s="57" t="n"/>
+      <x:c r="I6" s="57" t="n"/>
+      <x:c r="J6" s="57" t="n"/>
+      <x:c r="K6" s="57" t="n"/>
+      <x:c r="L6" s="57" t="n"/>
+      <x:c r="M6" s="57" t="n"/>
+      <x:c r="N6" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">BHXH</x:t>
         </x:is>
       </x:c>
-      <x:c r="O6" s="4" t="inlineStr">
+      <x:c r="O6" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">BHYT</x:t>
         </x:is>
       </x:c>
-      <x:c r="P6" s="4" t="inlineStr">
+      <x:c r="P6" s="42" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">BHTN</x:t>
         </x:is>
       </x:c>
-      <x:c r="Q6" s="10" t="n"/>
-      <x:c r="R6" s="10" t="n"/>
-      <x:c r="S6" s="10" t="n"/>
-      <x:c r="T6" s="10" t="n"/>
-      <x:c r="U6" s="10" t="n"/>
-      <x:c r="V6" s="10" t="n"/>
-      <x:c r="W6" s="10" t="n"/>
-      <x:c r="X6" s="10" t="n"/>
-      <x:c r="Y6" s="10" t="n"/>
-      <x:c r="Z6" s="10" t="n"/>
+      <x:c r="Q6" s="57" t="n"/>
+      <x:c r="R6" s="57" t="n"/>
+      <x:c r="S6" s="57" t="n"/>
+      <x:c r="T6" s="57" t="n"/>
+      <x:c r="U6" s="57" t="n"/>
+      <x:c r="V6" s="57" t="n"/>
+      <x:c r="W6" s="57" t="n"/>
+      <x:c r="X6" s="57" t="n"/>
+      <x:c r="Y6" s="57" t="n"/>
+      <x:c r="Z6" s="57" t="n"/>
     </x:row>
-    <x:row r="7" ht="54" customHeight="1">
-      <x:c r="A7" s="28" t="n">
+    <x:row r="7" ht="60" customHeight="1">
+      <x:c r="A7" s="32" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="29" t="inlineStr">
@@ -836,7 +894,7 @@
         </x:is>
       </x:c>
       <x:c r="G7" s="40" t="n"/>
-      <x:c r="H7" s="38" t="inlineStr">
+      <x:c r="H7" s="60" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">092086007417</x:t>
         </x:is>
@@ -846,8 +904,8 @@
           <x:t xml:space="preserve">Thạc sĩ</x:t>
         </x:is>
       </x:c>
-      <x:c r="J7" s="37" t="n"/>
-      <x:c r="K7" s="39" t="n"/>
+      <x:c r="J7" s="40" t="n"/>
+      <x:c r="K7" s="40" t="n"/>
       <x:c r="L7" s="36" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Không xác định</x:t>
@@ -865,19 +923,19 @@
       <x:c r="P7" s="41" t="n">
         <x:v>41379</x:v>
       </x:c>
-      <x:c r="Q7" s="34" t="n">
+      <x:c r="Q7" s="59" t="n">
         <x:v>26000000</x:v>
       </x:c>
-      <x:c r="R7" s="34" t="n">
+      <x:c r="R7" s="59" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="S7" s="32" t="n"/>
       <x:c r="T7" s="32" t="n"/>
-      <x:c r="U7" s="35" t="n"/>
-      <x:c r="V7" s="39" t="n"/>
-      <x:c r="W7" s="39" t="n"/>
-      <x:c r="X7" s="39" t="n"/>
-      <x:c r="Y7" s="39" t="n"/>
+      <x:c r="U7" s="32" t="n"/>
+      <x:c r="V7" s="40" t="n"/>
+      <x:c r="W7" s="40" t="n"/>
+      <x:c r="X7" s="40" t="n"/>
+      <x:c r="Y7" s="40" t="n"/>
       <x:c r="Z7" s="40" t="n"/>
     </x:row>
   </x:sheetData>

</xml_diff>